<commit_message>
feat: mejoras Excel import - duplicados, dieta Otro con detalle, modal scroll
</commit_message>
<xml_diff>
--- a/Lista de invitados ejemplo Events Boutique.xlsx
+++ b/Lista de invitados ejemplo Events Boutique.xlsx
@@ -1,32 +1,40 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://syngenta-my.sharepoint.com/personal/alejandro_lajnis_syngenta_com/Documents/Ale Personal/IA/RSVP app/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="12" documentId="8_{31A50830-2992-46F5-A763-CE04A31768A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8071F957-51BA-4AB2-A69F-2EC9F1E4C692}"/>
+  <xr:revisionPtr revIDLastSave="26" documentId="8_{31A50830-2992-46F5-A763-CE04A31768A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3568DFBB-4262-4CC4-AC23-759F2A01A146}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="importar lista invitados" sheetId="1" r:id="rId1"/>
     <sheet name="Instrucciones" sheetId="3" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="44">
   <si>
     <t>Invitación (Apellido)</t>
   </si>
@@ -136,9 +144,6 @@
     <t>Solo estos son campos obligatorios</t>
   </si>
   <si>
-    <t>juan@fernandez.com</t>
-  </si>
-  <si>
     <t>Mirta.gonzalez@gmail.com</t>
   </si>
   <si>
@@ -146,6 +151,21 @@
   </si>
   <si>
     <t>Emilia@duki.com</t>
+  </si>
+  <si>
+    <t>acompañante1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lajnis </t>
+  </si>
+  <si>
+    <t>Alejandro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fauda </t>
+  </si>
+  <si>
+    <t>Sofia</t>
   </si>
 </sst>
 </file>
@@ -233,25 +253,23 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -587,10 +605,32 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="525" row="3">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{8C611219-8C11-4461-BA2E-4CEAA18F264C}">
+  <we:reference id="wa200009404" version="1.0.0.8" store="es-ES" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="WA200009404" version="1.0.0.8" store="" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties>
+    <we:property name="claude.fileId" value="&quot;0c5a91e9-fb4d-423b-94fa-c0bab0304dcc&quot;"/>
+  </we:properties>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L346"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:L345"/>
+  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="17.5" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="17.33203125" bestFit="1" customWidth="1"/>
@@ -621,17 +661,17 @@
       <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="G1" t="s">
         <v>33</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="H1" t="s">
         <v>34</v>
       </c>
-      <c r="J1" s="9" t="s">
+      <c r="J1" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="K1" s="9"/>
-      <c r="L1" s="9"/>
+      <c r="K1" s="7"/>
+      <c r="L1" s="7"/>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
@@ -641,97 +681,91 @@
         <v>21</v>
       </c>
       <c r="C2" t="s">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="D2" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E2" t="s">
         <v>11</v>
       </c>
       <c r="F2" t="s">
-        <v>6</v>
-      </c>
-      <c r="G2" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="G2" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="H2" s="8">
-        <v>541169998887</v>
+      <c r="H2" s="6">
+        <v>541169954321</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="B3" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="C3" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="D3" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="E3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3" t="s">
+        <v>15</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="H3" s="6"/>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="C4" t="s">
+        <v>29</v>
+      </c>
+      <c r="D4" t="s">
+        <v>30</v>
+      </c>
+      <c r="E4" t="s">
         <v>11</v>
       </c>
-      <c r="F3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G3" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="H3" s="8">
-        <v>541169954321</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>27</v>
-      </c>
-      <c r="B4" t="s">
-        <v>28</v>
-      </c>
-      <c r="C4" t="s">
-        <v>27</v>
-      </c>
-      <c r="D4" t="s">
-        <v>28</v>
-      </c>
-      <c r="E4" t="s">
-        <v>10</v>
-      </c>
       <c r="F4" t="s">
-        <v>15</v>
-      </c>
-      <c r="G4" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="H4" s="8"/>
+        <v>16</v>
+      </c>
+      <c r="G4" s="4"/>
+      <c r="H4" s="6">
+        <v>541169991234</v>
+      </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B5" t="s">
-        <v>28</v>
-      </c>
-      <c r="C5" t="s">
-        <v>29</v>
-      </c>
-      <c r="D5" t="s">
-        <v>30</v>
+        <v>32</v>
+      </c>
+      <c r="C5" t="str">
+        <f>IF(A4="",A5,"")</f>
+        <v>Mernes</v>
+      </c>
+      <c r="D5" t="str">
+        <f>IF(B4="",B5,"")</f>
+        <v>Emilia</v>
       </c>
       <c r="E5" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="F5" t="s">
-        <v>16</v>
-      </c>
-      <c r="G5" s="6"/>
-      <c r="H5" s="8">
-        <v>541169991234</v>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="H5" s="6"/>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
@@ -741,1053 +775,1064 @@
         <v>32</v>
       </c>
       <c r="C6" t="s">
-        <v>31</v>
-      </c>
-      <c r="D6" t="s">
-        <v>32</v>
-      </c>
-      <c r="E6" t="s">
-        <v>7</v>
-      </c>
-      <c r="F6" t="s">
-        <v>6</v>
-      </c>
-      <c r="G6" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="H6" s="8"/>
+      <c r="D6" t="str">
+        <f>IF(B5="",B6,"")</f>
+        <v/>
+      </c>
+      <c r="H6" s="6"/>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="H7" s="8"/>
+      <c r="A7" t="s">
+        <v>40</v>
+      </c>
+      <c r="B7" t="s">
+        <v>41</v>
+      </c>
+      <c r="E7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F7" t="s">
+        <v>16</v>
+      </c>
+      <c r="H7" s="6"/>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="H8" s="8"/>
+      <c r="A8" t="s">
+        <v>42</v>
+      </c>
+      <c r="B8" t="s">
+        <v>43</v>
+      </c>
+      <c r="E8" t="s">
+        <v>11</v>
+      </c>
+      <c r="F8" t="s">
+        <v>16</v>
+      </c>
+      <c r="H8" s="6"/>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="H9" s="8"/>
+      <c r="H9" s="6"/>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="H10" s="8"/>
+      <c r="H10" s="6"/>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="H11" s="8"/>
+      <c r="H11" s="6"/>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="H12" s="8"/>
+      <c r="H12" s="6"/>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="H13" s="8"/>
+      <c r="H13" s="6"/>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="H14" s="8"/>
+      <c r="H14" s="6"/>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="H15" s="8"/>
+      <c r="H15" s="6"/>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="C16" s="4"/>
-      <c r="H16" s="8"/>
+      <c r="H16" s="6"/>
     </row>
     <row r="17" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H17" s="8"/>
+      <c r="H17" s="6"/>
     </row>
     <row r="18" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H18" s="8"/>
+      <c r="H18" s="6"/>
     </row>
     <row r="19" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H19" s="8"/>
+      <c r="H19" s="6"/>
     </row>
     <row r="20" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H20" s="8"/>
+      <c r="H20" s="6"/>
     </row>
     <row r="21" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H21" s="8"/>
+      <c r="H21" s="6"/>
     </row>
     <row r="22" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H22" s="8"/>
+      <c r="H22" s="6"/>
     </row>
     <row r="23" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H23" s="8"/>
+      <c r="H23" s="6"/>
     </row>
     <row r="24" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H24" s="8"/>
+      <c r="H24" s="6"/>
     </row>
     <row r="25" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H25" s="8"/>
+      <c r="H25" s="6"/>
     </row>
     <row r="26" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H26" s="8"/>
+      <c r="H26" s="6"/>
     </row>
     <row r="27" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H27" s="8"/>
+      <c r="H27" s="6"/>
     </row>
     <row r="28" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H28" s="8"/>
+      <c r="H28" s="6"/>
     </row>
     <row r="29" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H29" s="8"/>
+      <c r="H29" s="6"/>
     </row>
     <row r="30" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H30" s="8"/>
+      <c r="H30" s="6"/>
     </row>
     <row r="31" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H31" s="8"/>
+      <c r="H31" s="6"/>
     </row>
     <row r="32" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H32" s="8"/>
+      <c r="H32" s="6"/>
     </row>
     <row r="33" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H33" s="8"/>
+      <c r="H33" s="6"/>
     </row>
     <row r="34" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H34" s="8"/>
+      <c r="H34" s="6"/>
     </row>
     <row r="35" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H35" s="8"/>
+      <c r="H35" s="6"/>
     </row>
     <row r="36" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H36" s="8"/>
+      <c r="H36" s="6"/>
     </row>
     <row r="37" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H37" s="8"/>
+      <c r="H37" s="6"/>
     </row>
     <row r="38" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H38" s="8"/>
+      <c r="H38" s="6"/>
     </row>
     <row r="39" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H39" s="8"/>
+      <c r="H39" s="6"/>
     </row>
     <row r="40" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H40" s="8"/>
+      <c r="H40" s="6"/>
     </row>
     <row r="41" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H41" s="8"/>
+      <c r="H41" s="6"/>
     </row>
     <row r="42" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H42" s="8"/>
+      <c r="H42" s="6"/>
     </row>
     <row r="43" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H43" s="8"/>
+      <c r="H43" s="6"/>
     </row>
     <row r="44" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H44" s="8"/>
+      <c r="H44" s="6"/>
     </row>
     <row r="45" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H45" s="8"/>
+      <c r="H45" s="6"/>
     </row>
     <row r="46" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H46" s="8"/>
+      <c r="H46" s="6"/>
     </row>
     <row r="47" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H47" s="8"/>
+      <c r="H47" s="6"/>
     </row>
     <row r="48" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H48" s="8"/>
+      <c r="H48" s="6"/>
     </row>
     <row r="49" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H49" s="8"/>
+      <c r="H49" s="6"/>
     </row>
     <row r="50" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H50" s="8"/>
+      <c r="H50" s="6"/>
     </row>
     <row r="51" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H51" s="8"/>
+      <c r="H51" s="6"/>
     </row>
     <row r="52" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H52" s="8"/>
+      <c r="H52" s="6"/>
     </row>
     <row r="53" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H53" s="8"/>
+      <c r="H53" s="6"/>
     </row>
     <row r="54" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H54" s="8"/>
+      <c r="H54" s="6"/>
     </row>
     <row r="55" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H55" s="8"/>
+      <c r="H55" s="6"/>
     </row>
     <row r="56" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H56" s="8"/>
+      <c r="H56" s="6"/>
     </row>
     <row r="57" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H57" s="8"/>
+      <c r="H57" s="6"/>
     </row>
     <row r="58" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H58" s="8"/>
+      <c r="H58" s="6"/>
     </row>
     <row r="59" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H59" s="8"/>
+      <c r="H59" s="6"/>
     </row>
     <row r="60" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H60" s="8"/>
+      <c r="H60" s="6"/>
     </row>
     <row r="61" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H61" s="8"/>
+      <c r="H61" s="6"/>
     </row>
     <row r="62" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H62" s="8"/>
+      <c r="H62" s="6"/>
     </row>
     <row r="63" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H63" s="8"/>
+      <c r="H63" s="6"/>
     </row>
     <row r="64" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H64" s="8"/>
+      <c r="H64" s="6"/>
     </row>
     <row r="65" spans="6:8" x14ac:dyDescent="0.35">
-      <c r="H65" s="8"/>
+      <c r="H65" s="6"/>
     </row>
     <row r="66" spans="6:8" x14ac:dyDescent="0.35">
-      <c r="H66" s="8"/>
+      <c r="H66" s="6"/>
     </row>
     <row r="67" spans="6:8" x14ac:dyDescent="0.35">
-      <c r="H67" s="8"/>
+      <c r="H67" s="6"/>
     </row>
     <row r="68" spans="6:8" x14ac:dyDescent="0.35">
-      <c r="H68" s="8"/>
+      <c r="H68" s="6"/>
     </row>
     <row r="69" spans="6:8" x14ac:dyDescent="0.35">
-      <c r="H69" s="8"/>
+      <c r="H69" s="6"/>
     </row>
     <row r="70" spans="6:8" x14ac:dyDescent="0.35">
-      <c r="H70" s="8"/>
+      <c r="H70" s="6"/>
     </row>
     <row r="71" spans="6:8" x14ac:dyDescent="0.35">
-      <c r="H71" s="8"/>
+      <c r="H71" s="6"/>
     </row>
     <row r="72" spans="6:8" x14ac:dyDescent="0.35">
-      <c r="H72" s="8"/>
+      <c r="H72" s="6"/>
     </row>
     <row r="73" spans="6:8" x14ac:dyDescent="0.35">
-      <c r="H73" s="8"/>
+      <c r="H73" s="6"/>
     </row>
     <row r="74" spans="6:8" x14ac:dyDescent="0.35">
-      <c r="H74" s="8"/>
+      <c r="H74" s="6"/>
     </row>
     <row r="75" spans="6:8" x14ac:dyDescent="0.35">
-      <c r="H75" s="8"/>
+      <c r="H75" s="6"/>
     </row>
     <row r="76" spans="6:8" x14ac:dyDescent="0.35">
-      <c r="H76" s="8"/>
+      <c r="H76" s="6"/>
     </row>
     <row r="77" spans="6:8" x14ac:dyDescent="0.35">
-      <c r="H77" s="8"/>
+      <c r="F77" s="1"/>
+      <c r="H77" s="6"/>
     </row>
     <row r="78" spans="6:8" x14ac:dyDescent="0.35">
-      <c r="F78" s="1"/>
-      <c r="H78" s="8"/>
+      <c r="H78" s="6"/>
     </row>
     <row r="79" spans="6:8" x14ac:dyDescent="0.35">
-      <c r="H79" s="8"/>
+      <c r="H79" s="6"/>
     </row>
     <row r="80" spans="6:8" x14ac:dyDescent="0.35">
-      <c r="H80" s="8"/>
+      <c r="H80" s="6"/>
     </row>
     <row r="81" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H81" s="8"/>
+      <c r="H81" s="6"/>
     </row>
     <row r="82" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H82" s="8"/>
+      <c r="H82" s="6"/>
     </row>
     <row r="83" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H83" s="8"/>
+      <c r="H83" s="6"/>
     </row>
     <row r="84" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H84" s="8"/>
+      <c r="H84" s="6"/>
     </row>
     <row r="85" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H85" s="8"/>
+      <c r="H85" s="6"/>
     </row>
     <row r="86" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H86" s="8"/>
+      <c r="H86" s="6"/>
     </row>
     <row r="87" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H87" s="8"/>
+      <c r="H87" s="6"/>
     </row>
     <row r="88" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H88" s="8"/>
+      <c r="H88" s="6"/>
     </row>
     <row r="89" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H89" s="8"/>
+      <c r="H89" s="6"/>
     </row>
     <row r="90" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H90" s="8"/>
+      <c r="H90" s="6"/>
     </row>
     <row r="91" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H91" s="8"/>
+      <c r="H91" s="6"/>
     </row>
     <row r="92" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H92" s="8"/>
+      <c r="H92" s="6"/>
     </row>
     <row r="93" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H93" s="8"/>
+      <c r="H93" s="6"/>
     </row>
     <row r="94" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H94" s="8"/>
+      <c r="H94" s="6"/>
     </row>
     <row r="95" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H95" s="8"/>
+      <c r="H95" s="6"/>
     </row>
     <row r="96" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H96" s="8"/>
+      <c r="H96" s="6"/>
     </row>
     <row r="97" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H97" s="8"/>
+      <c r="H97" s="6"/>
     </row>
     <row r="98" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H98" s="8"/>
+      <c r="H98" s="6"/>
     </row>
     <row r="99" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H99" s="8"/>
+      <c r="H99" s="6"/>
     </row>
     <row r="100" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H100" s="8"/>
+      <c r="H100" s="6"/>
     </row>
     <row r="101" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H101" s="8"/>
+      <c r="H101" s="6"/>
     </row>
     <row r="102" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H102" s="8"/>
+      <c r="H102" s="6"/>
     </row>
     <row r="103" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H103" s="8"/>
+      <c r="H103" s="6"/>
     </row>
     <row r="104" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H104" s="8"/>
+      <c r="H104" s="6"/>
     </row>
     <row r="105" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H105" s="8"/>
+      <c r="H105" s="6"/>
     </row>
     <row r="106" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H106" s="8"/>
+      <c r="H106" s="6"/>
     </row>
     <row r="107" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H107" s="8"/>
+      <c r="H107" s="6"/>
     </row>
     <row r="108" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H108" s="8"/>
+      <c r="H108" s="6"/>
     </row>
     <row r="109" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H109" s="8"/>
+      <c r="H109" s="6"/>
     </row>
     <row r="110" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H110" s="8"/>
+      <c r="H110" s="6"/>
     </row>
     <row r="111" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H111" s="8"/>
+      <c r="H111" s="6"/>
     </row>
     <row r="112" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H112" s="8"/>
+      <c r="H112" s="6"/>
     </row>
     <row r="113" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H113" s="8"/>
+      <c r="H113" s="6"/>
     </row>
     <row r="114" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H114" s="8"/>
+      <c r="H114" s="6"/>
     </row>
     <row r="115" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H115" s="8"/>
+      <c r="H115" s="6"/>
     </row>
     <row r="116" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H116" s="8"/>
+      <c r="H116" s="6"/>
     </row>
     <row r="117" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H117" s="8"/>
+      <c r="H117" s="6"/>
     </row>
     <row r="118" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H118" s="8"/>
+      <c r="H118" s="6"/>
     </row>
     <row r="119" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H119" s="8"/>
+      <c r="H119" s="6"/>
     </row>
     <row r="120" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H120" s="8"/>
+      <c r="H120" s="6"/>
     </row>
     <row r="121" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H121" s="8"/>
+      <c r="H121" s="6"/>
     </row>
     <row r="122" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H122" s="8"/>
+      <c r="H122" s="6"/>
     </row>
     <row r="123" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H123" s="8"/>
+      <c r="H123" s="6"/>
     </row>
     <row r="124" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H124" s="8"/>
+      <c r="H124" s="6"/>
     </row>
     <row r="125" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H125" s="8"/>
+      <c r="H125" s="6"/>
     </row>
     <row r="126" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H126" s="8"/>
+      <c r="H126" s="6"/>
     </row>
     <row r="127" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H127" s="8"/>
+      <c r="H127" s="6"/>
     </row>
     <row r="128" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H128" s="8"/>
+      <c r="H128" s="6"/>
     </row>
     <row r="129" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H129" s="8"/>
+      <c r="H129" s="6"/>
     </row>
     <row r="130" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H130" s="8"/>
+      <c r="H130" s="6"/>
     </row>
     <row r="131" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H131" s="8"/>
+      <c r="H131" s="6"/>
     </row>
     <row r="132" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H132" s="8"/>
+      <c r="H132" s="6"/>
     </row>
     <row r="133" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H133" s="8"/>
+      <c r="H133" s="6"/>
     </row>
     <row r="134" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H134" s="8"/>
+      <c r="H134" s="6"/>
     </row>
     <row r="135" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H135" s="8"/>
+      <c r="H135" s="6"/>
     </row>
     <row r="136" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H136" s="8"/>
+      <c r="H136" s="6"/>
     </row>
     <row r="137" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H137" s="8"/>
+      <c r="H137" s="6"/>
     </row>
     <row r="138" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H138" s="8"/>
+      <c r="H138" s="6"/>
     </row>
     <row r="139" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H139" s="8"/>
+      <c r="H139" s="6"/>
     </row>
     <row r="140" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H140" s="8"/>
+      <c r="H140" s="6"/>
     </row>
     <row r="141" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H141" s="8"/>
+      <c r="H141" s="6"/>
     </row>
     <row r="142" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H142" s="8"/>
+      <c r="H142" s="6"/>
     </row>
     <row r="143" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H143" s="8"/>
+      <c r="H143" s="6"/>
     </row>
     <row r="144" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H144" s="8"/>
+      <c r="H144" s="6"/>
     </row>
     <row r="145" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H145" s="8"/>
+      <c r="H145" s="6"/>
     </row>
     <row r="146" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H146" s="8"/>
+      <c r="H146" s="6"/>
     </row>
     <row r="147" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H147" s="8"/>
+      <c r="H147" s="6"/>
     </row>
     <row r="148" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H148" s="8"/>
+      <c r="H148" s="6"/>
     </row>
     <row r="149" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H149" s="8"/>
+      <c r="H149" s="6"/>
     </row>
     <row r="150" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H150" s="8"/>
+      <c r="H150" s="6"/>
     </row>
     <row r="151" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H151" s="8"/>
+      <c r="H151" s="6"/>
     </row>
     <row r="152" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H152" s="8"/>
+      <c r="H152" s="6"/>
     </row>
     <row r="153" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H153" s="8"/>
+      <c r="H153" s="6"/>
     </row>
     <row r="154" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H154" s="8"/>
+      <c r="H154" s="6"/>
     </row>
     <row r="155" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H155" s="8"/>
+      <c r="H155" s="6"/>
     </row>
     <row r="156" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H156" s="8"/>
+      <c r="H156" s="6"/>
     </row>
     <row r="157" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H157" s="8"/>
+      <c r="H157" s="6"/>
     </row>
     <row r="158" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H158" s="8"/>
+      <c r="H158" s="6"/>
     </row>
     <row r="159" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H159" s="8"/>
+      <c r="H159" s="6"/>
     </row>
     <row r="160" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H160" s="8"/>
+      <c r="H160" s="6"/>
     </row>
     <row r="161" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H161" s="8"/>
+      <c r="H161" s="6"/>
     </row>
     <row r="162" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H162" s="8"/>
+      <c r="H162" s="6"/>
     </row>
     <row r="163" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H163" s="8"/>
+      <c r="H163" s="6"/>
     </row>
     <row r="164" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H164" s="8"/>
+      <c r="H164" s="6"/>
     </row>
     <row r="165" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H165" s="8"/>
+      <c r="H165" s="6"/>
     </row>
     <row r="166" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H166" s="8"/>
+      <c r="H166" s="6"/>
     </row>
     <row r="167" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H167" s="8"/>
+      <c r="H167" s="6"/>
     </row>
     <row r="168" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H168" s="8"/>
+      <c r="H168" s="6"/>
     </row>
     <row r="169" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H169" s="8"/>
+      <c r="H169" s="6"/>
     </row>
     <row r="170" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H170" s="8"/>
+      <c r="H170" s="6"/>
     </row>
     <row r="171" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H171" s="8"/>
+      <c r="H171" s="6"/>
     </row>
     <row r="172" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H172" s="8"/>
+      <c r="H172" s="6"/>
     </row>
     <row r="173" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H173" s="8"/>
+      <c r="H173" s="6"/>
     </row>
     <row r="174" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H174" s="8"/>
+      <c r="H174" s="6"/>
     </row>
     <row r="175" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H175" s="8"/>
+      <c r="H175" s="6"/>
     </row>
     <row r="176" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H176" s="8"/>
+      <c r="H176" s="6"/>
     </row>
     <row r="177" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H177" s="8"/>
+      <c r="H177" s="6"/>
     </row>
     <row r="178" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H178" s="8"/>
+      <c r="H178" s="6"/>
     </row>
     <row r="179" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H179" s="8"/>
+      <c r="H179" s="6"/>
     </row>
     <row r="180" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H180" s="8"/>
+      <c r="H180" s="6"/>
     </row>
     <row r="181" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H181" s="8"/>
+      <c r="H181" s="6"/>
     </row>
     <row r="182" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H182" s="8"/>
+      <c r="H182" s="6"/>
     </row>
     <row r="183" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H183" s="8"/>
+      <c r="H183" s="6"/>
     </row>
     <row r="184" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H184" s="8"/>
+      <c r="H184" s="6"/>
     </row>
     <row r="185" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H185" s="8"/>
+      <c r="H185" s="6"/>
     </row>
     <row r="186" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H186" s="8"/>
+      <c r="H186" s="6"/>
     </row>
     <row r="187" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H187" s="8"/>
+      <c r="H187" s="6"/>
     </row>
     <row r="188" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H188" s="8"/>
+      <c r="H188" s="6"/>
     </row>
     <row r="189" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H189" s="8"/>
+      <c r="H189" s="6"/>
     </row>
     <row r="190" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H190" s="8"/>
+      <c r="H190" s="6"/>
     </row>
     <row r="191" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H191" s="8"/>
+      <c r="H191" s="6"/>
     </row>
     <row r="192" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H192" s="8"/>
+      <c r="H192" s="6"/>
     </row>
     <row r="193" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H193" s="8"/>
+      <c r="H193" s="6"/>
     </row>
     <row r="194" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H194" s="8"/>
+      <c r="H194" s="6"/>
     </row>
     <row r="195" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H195" s="8"/>
+      <c r="H195" s="6"/>
     </row>
     <row r="196" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H196" s="8"/>
+      <c r="H196" s="6"/>
     </row>
     <row r="197" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H197" s="8"/>
+      <c r="H197" s="6"/>
     </row>
     <row r="198" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H198" s="8"/>
+      <c r="H198" s="6"/>
     </row>
     <row r="199" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H199" s="8"/>
+      <c r="H199" s="6"/>
     </row>
     <row r="200" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H200" s="8"/>
+      <c r="H200" s="6"/>
     </row>
     <row r="201" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H201" s="8"/>
+      <c r="H201" s="6"/>
     </row>
     <row r="202" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H202" s="8"/>
+      <c r="H202" s="6"/>
     </row>
     <row r="203" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H203" s="8"/>
+      <c r="H203" s="6"/>
     </row>
     <row r="204" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H204" s="8"/>
+      <c r="H204" s="6"/>
     </row>
     <row r="205" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H205" s="8"/>
+      <c r="H205" s="6"/>
     </row>
     <row r="206" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H206" s="8"/>
+      <c r="H206" s="6"/>
     </row>
     <row r="207" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H207" s="8"/>
+      <c r="H207" s="6"/>
     </row>
     <row r="208" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H208" s="8"/>
+      <c r="H208" s="6"/>
     </row>
     <row r="209" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H209" s="8"/>
+      <c r="H209" s="6"/>
     </row>
     <row r="210" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H210" s="8"/>
+      <c r="H210" s="6"/>
     </row>
     <row r="211" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H211" s="8"/>
+      <c r="H211" s="6"/>
     </row>
     <row r="212" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H212" s="8"/>
+      <c r="H212" s="6"/>
     </row>
     <row r="213" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H213" s="8"/>
+      <c r="H213" s="6"/>
     </row>
     <row r="214" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H214" s="8"/>
+      <c r="H214" s="6"/>
     </row>
     <row r="215" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H215" s="8"/>
+      <c r="H215" s="6"/>
     </row>
     <row r="216" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H216" s="8"/>
+      <c r="H216" s="6"/>
     </row>
     <row r="217" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H217" s="8"/>
+      <c r="H217" s="6"/>
     </row>
     <row r="218" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H218" s="8"/>
+      <c r="H218" s="6"/>
     </row>
     <row r="219" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H219" s="8"/>
+      <c r="H219" s="6"/>
     </row>
     <row r="220" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H220" s="8"/>
+      <c r="H220" s="6"/>
     </row>
     <row r="221" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H221" s="8"/>
+      <c r="H221" s="6"/>
     </row>
     <row r="222" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H222" s="8"/>
+      <c r="H222" s="6"/>
     </row>
     <row r="223" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H223" s="8"/>
+      <c r="H223" s="6"/>
     </row>
     <row r="224" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H224" s="8"/>
+      <c r="H224" s="6"/>
     </row>
     <row r="225" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H225" s="8"/>
+      <c r="H225" s="6"/>
     </row>
     <row r="226" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H226" s="8"/>
+      <c r="H226" s="6"/>
     </row>
     <row r="227" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H227" s="8"/>
+      <c r="H227" s="6"/>
     </row>
     <row r="228" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H228" s="8"/>
+      <c r="H228" s="6"/>
     </row>
     <row r="229" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H229" s="8"/>
+      <c r="H229" s="6"/>
     </row>
     <row r="230" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H230" s="8"/>
+      <c r="H230" s="6"/>
     </row>
     <row r="231" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H231" s="8"/>
+      <c r="H231" s="6"/>
     </row>
     <row r="232" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H232" s="8"/>
+      <c r="H232" s="6"/>
     </row>
     <row r="233" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H233" s="8"/>
+      <c r="H233" s="6"/>
     </row>
     <row r="234" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H234" s="8"/>
+      <c r="H234" s="6"/>
     </row>
     <row r="235" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H235" s="8"/>
+      <c r="H235" s="6"/>
     </row>
     <row r="236" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H236" s="8"/>
+      <c r="H236" s="6"/>
     </row>
     <row r="237" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H237" s="8"/>
+      <c r="H237" s="6"/>
     </row>
     <row r="238" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H238" s="8"/>
+      <c r="H238" s="6"/>
     </row>
     <row r="239" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H239" s="8"/>
+      <c r="H239" s="6"/>
     </row>
     <row r="240" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H240" s="8"/>
+      <c r="H240" s="6"/>
     </row>
     <row r="241" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H241" s="8"/>
+      <c r="H241" s="6"/>
     </row>
     <row r="242" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H242" s="8"/>
+      <c r="H242" s="6"/>
     </row>
     <row r="243" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H243" s="8"/>
+      <c r="H243" s="6"/>
     </row>
     <row r="244" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H244" s="8"/>
+      <c r="H244" s="6"/>
     </row>
     <row r="245" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H245" s="8"/>
+      <c r="H245" s="6"/>
     </row>
     <row r="246" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H246" s="8"/>
+      <c r="H246" s="6"/>
     </row>
     <row r="247" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H247" s="8"/>
+      <c r="H247" s="6"/>
     </row>
     <row r="248" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H248" s="8"/>
+      <c r="H248" s="6"/>
     </row>
     <row r="249" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H249" s="8"/>
+      <c r="H249" s="6"/>
     </row>
     <row r="250" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H250" s="8"/>
+      <c r="H250" s="6"/>
     </row>
     <row r="251" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H251" s="8"/>
+      <c r="H251" s="6"/>
     </row>
     <row r="252" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H252" s="8"/>
+      <c r="H252" s="6"/>
     </row>
     <row r="253" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H253" s="8"/>
+      <c r="H253" s="6"/>
     </row>
     <row r="254" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H254" s="8"/>
+      <c r="H254" s="6"/>
     </row>
     <row r="255" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H255" s="8"/>
+      <c r="H255" s="6"/>
     </row>
     <row r="256" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H256" s="8"/>
+      <c r="H256" s="6"/>
     </row>
     <row r="257" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H257" s="8"/>
+      <c r="H257" s="6"/>
     </row>
     <row r="258" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H258" s="8"/>
+      <c r="H258" s="6"/>
     </row>
     <row r="259" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H259" s="8"/>
+      <c r="H259" s="6"/>
     </row>
     <row r="260" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H260" s="8"/>
+      <c r="H260" s="6"/>
     </row>
     <row r="261" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H261" s="8"/>
+      <c r="H261" s="6"/>
     </row>
     <row r="262" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H262" s="8"/>
+      <c r="H262" s="6"/>
     </row>
     <row r="263" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H263" s="8"/>
+      <c r="H263" s="6"/>
     </row>
     <row r="264" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H264" s="8"/>
+      <c r="H264" s="6"/>
     </row>
     <row r="265" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H265" s="8"/>
+      <c r="H265" s="6"/>
     </row>
     <row r="266" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H266" s="8"/>
+      <c r="H266" s="6"/>
     </row>
     <row r="267" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H267" s="8"/>
+      <c r="H267" s="6"/>
     </row>
     <row r="268" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H268" s="8"/>
+      <c r="H268" s="6"/>
     </row>
     <row r="269" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H269" s="8"/>
+      <c r="H269" s="6"/>
     </row>
     <row r="270" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H270" s="8"/>
+      <c r="H270" s="6"/>
     </row>
     <row r="271" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H271" s="8"/>
+      <c r="H271" s="6"/>
     </row>
     <row r="272" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H272" s="8"/>
+      <c r="H272" s="6"/>
     </row>
     <row r="273" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H273" s="8"/>
+      <c r="H273" s="6"/>
     </row>
     <row r="274" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H274" s="8"/>
+      <c r="H274" s="6"/>
     </row>
     <row r="275" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H275" s="8"/>
+      <c r="H275" s="6"/>
     </row>
     <row r="276" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H276" s="8"/>
+      <c r="H276" s="6"/>
     </row>
     <row r="277" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H277" s="8"/>
+      <c r="H277" s="6"/>
     </row>
     <row r="278" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H278" s="8"/>
+      <c r="H278" s="6"/>
     </row>
     <row r="279" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H279" s="8"/>
+      <c r="H279" s="6"/>
     </row>
     <row r="280" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H280" s="8"/>
+      <c r="H280" s="6"/>
     </row>
     <row r="281" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H281" s="8"/>
+      <c r="H281" s="6"/>
     </row>
     <row r="282" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H282" s="8"/>
+      <c r="H282" s="6"/>
     </row>
     <row r="283" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H283" s="8"/>
+      <c r="H283" s="6"/>
     </row>
     <row r="284" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H284" s="8"/>
+      <c r="H284" s="6"/>
     </row>
     <row r="285" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H285" s="8"/>
+      <c r="H285" s="6"/>
     </row>
     <row r="286" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H286" s="8"/>
+      <c r="H286" s="6"/>
     </row>
     <row r="287" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H287" s="8"/>
+      <c r="H287" s="6"/>
     </row>
     <row r="288" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H288" s="8"/>
+      <c r="H288" s="6"/>
     </row>
     <row r="289" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H289" s="8"/>
+      <c r="H289" s="6"/>
     </row>
     <row r="290" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H290" s="8"/>
+      <c r="H290" s="6"/>
     </row>
     <row r="291" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H291" s="8"/>
+      <c r="H291" s="6"/>
     </row>
     <row r="292" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H292" s="8"/>
+      <c r="H292" s="6"/>
     </row>
     <row r="293" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H293" s="8"/>
+      <c r="H293" s="6"/>
     </row>
     <row r="294" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H294" s="8"/>
+      <c r="H294" s="6"/>
     </row>
     <row r="295" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H295" s="8"/>
+      <c r="H295" s="6"/>
     </row>
     <row r="296" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H296" s="8"/>
+      <c r="H296" s="6"/>
     </row>
     <row r="297" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H297" s="8"/>
+      <c r="H297" s="6"/>
     </row>
     <row r="298" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H298" s="8"/>
+      <c r="H298" s="6"/>
     </row>
     <row r="299" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H299" s="8"/>
+      <c r="H299" s="6"/>
     </row>
     <row r="300" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H300" s="8"/>
+      <c r="H300" s="6"/>
     </row>
     <row r="301" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H301" s="8"/>
+      <c r="H301" s="6"/>
     </row>
     <row r="302" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H302" s="8"/>
+      <c r="H302" s="6"/>
     </row>
     <row r="303" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H303" s="8"/>
+      <c r="H303" s="6"/>
     </row>
     <row r="304" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H304" s="8"/>
+      <c r="H304" s="6"/>
     </row>
     <row r="305" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H305" s="8"/>
+      <c r="H305" s="6"/>
     </row>
     <row r="306" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H306" s="8"/>
+      <c r="H306" s="6"/>
     </row>
     <row r="307" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H307" s="8"/>
+      <c r="H307" s="6"/>
     </row>
     <row r="308" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H308" s="8"/>
+      <c r="H308" s="6"/>
     </row>
     <row r="309" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H309" s="8"/>
+      <c r="H309" s="6"/>
     </row>
     <row r="310" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H310" s="8"/>
+      <c r="H310" s="6"/>
     </row>
     <row r="311" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H311" s="8"/>
+      <c r="H311" s="6"/>
     </row>
     <row r="312" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H312" s="8"/>
+      <c r="H312" s="6"/>
     </row>
     <row r="313" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H313" s="8"/>
+      <c r="H313" s="6"/>
     </row>
     <row r="314" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H314" s="8"/>
+      <c r="H314" s="6"/>
     </row>
     <row r="315" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H315" s="8"/>
+      <c r="H315" s="6"/>
     </row>
     <row r="316" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H316" s="8"/>
+      <c r="H316" s="6"/>
     </row>
     <row r="317" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H317" s="8"/>
+      <c r="H317" s="6"/>
     </row>
     <row r="318" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H318" s="8"/>
+      <c r="H318" s="6"/>
     </row>
     <row r="319" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H319" s="8"/>
+      <c r="H319" s="6"/>
     </row>
     <row r="320" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H320" s="8"/>
+      <c r="H320" s="6"/>
     </row>
     <row r="321" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H321" s="8"/>
+      <c r="H321" s="6"/>
     </row>
     <row r="322" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H322" s="8"/>
+      <c r="H322" s="6"/>
     </row>
     <row r="323" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H323" s="8"/>
+      <c r="H323" s="6"/>
     </row>
     <row r="324" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H324" s="8"/>
+      <c r="H324" s="6"/>
     </row>
     <row r="325" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H325" s="8"/>
+      <c r="H325" s="6"/>
     </row>
     <row r="326" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H326" s="8"/>
+      <c r="H326" s="6"/>
     </row>
     <row r="327" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H327" s="8"/>
+      <c r="H327" s="6"/>
     </row>
     <row r="328" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H328" s="8"/>
+      <c r="H328" s="6"/>
     </row>
     <row r="329" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H329" s="8"/>
+      <c r="H329" s="6"/>
     </row>
     <row r="330" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H330" s="8"/>
+      <c r="H330" s="6"/>
     </row>
     <row r="331" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H331" s="8"/>
+      <c r="H331" s="6"/>
     </row>
     <row r="332" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H332" s="8"/>
+      <c r="H332" s="6"/>
     </row>
     <row r="333" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H333" s="8"/>
+      <c r="H333" s="6"/>
     </row>
     <row r="334" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H334" s="8"/>
+      <c r="H334" s="6"/>
     </row>
     <row r="335" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H335" s="8"/>
+      <c r="H335" s="6"/>
     </row>
     <row r="336" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H336" s="8"/>
+      <c r="H336" s="6"/>
     </row>
     <row r="337" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H337" s="8"/>
+      <c r="H337" s="6"/>
     </row>
     <row r="338" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H338" s="8"/>
+      <c r="H338" s="6"/>
     </row>
     <row r="339" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H339" s="8"/>
+      <c r="H339" s="6"/>
     </row>
     <row r="340" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H340" s="8"/>
+      <c r="H340" s="6"/>
     </row>
     <row r="341" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H341" s="8"/>
+      <c r="H341" s="6"/>
     </row>
     <row r="342" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H342" s="8"/>
+      <c r="H342" s="6"/>
     </row>
     <row r="343" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H343" s="8"/>
+      <c r="H343" s="6"/>
     </row>
     <row r="344" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H344" s="8"/>
+      <c r="H344" s="6"/>
     </row>
     <row r="345" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H345" s="8"/>
-    </row>
-    <row r="346" spans="8:8" x14ac:dyDescent="0.35">
-      <c r="H346" s="8"/>
+      <c r="H345" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="J1:L1"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="G2" r:id="rId1" xr:uid="{8AF6A04B-B363-40A7-A4E9-10ADFACC1E68}"/>
-    <hyperlink ref="G3" r:id="rId2" xr:uid="{A38FE408-4272-40B3-803F-F1FDE2495CB0}"/>
-    <hyperlink ref="G4" r:id="rId3" xr:uid="{1C09D097-983B-4DC5-965C-052B318757C0}"/>
-    <hyperlink ref="G6" r:id="rId4" xr:uid="{1797E710-D6AA-45D2-B79B-DE037EAD4446}"/>
+    <hyperlink ref="G2" r:id="rId1" xr:uid="{A38FE408-4272-40B3-803F-F1FDE2495CB0}"/>
+    <hyperlink ref="G3" r:id="rId2" xr:uid="{1C09D097-983B-4DC5-965C-052B318757C0}"/>
+    <hyperlink ref="G5" r:id="rId3" xr:uid="{1797E710-D6AA-45D2-B79B-DE037EAD4446}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
@@ -1800,13 +1845,13 @@
           <x14:formula1>
             <xm:f>Instrucciones!$AC$2:$AC$7</xm:f>
           </x14:formula1>
-          <xm:sqref>E2:E91</xm:sqref>
+          <xm:sqref>E2:E90</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{BD3EA716-187E-4E8D-AD24-6E0BA0BEF0DE}">
           <x14:formula1>
             <xm:f>Instrucciones!$AD$2:$AD$5</xm:f>
           </x14:formula1>
-          <xm:sqref>F2:F91</xm:sqref>
+          <xm:sqref>F2:F90</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -1817,19 +1862,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BDC79005-B21E-48CC-BFB9-5EB91A3C02C7}">
   <dimension ref="A1:AD9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:30" x14ac:dyDescent="0.35">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
-      <c r="F1" s="10"/>
-      <c r="G1" s="10"/>
-      <c r="H1" s="10"/>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="8"/>
+      <c r="H1" s="8"/>
       <c r="AC1" s="3" t="s">
         <v>4</v>
       </c>
@@ -1838,14 +1883,14 @@
       </c>
     </row>
     <row r="2" spans="1:30" x14ac:dyDescent="0.35">
-      <c r="A2" s="10"/>
-      <c r="B2" s="10"/>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10"/>
-      <c r="F2" s="10"/>
-      <c r="G2" s="10"/>
-      <c r="H2" s="10"/>
+      <c r="A2" s="8"/>
+      <c r="B2" s="8"/>
+      <c r="C2" s="8"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="8"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="8"/>
+      <c r="H2" s="8"/>
       <c r="AC2" s="3" t="s">
         <v>11</v>
       </c>
@@ -1907,7 +1952,7 @@
       </c>
     </row>
     <row r="9" spans="1:30" x14ac:dyDescent="0.35">
-      <c r="A9" s="4" t="s">
+      <c r="A9" t="s">
         <v>24</v>
       </c>
     </row>
@@ -1921,6 +1966,6 @@
 
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
-  <clbl:label id="{06219a4a-a835-44d5-afaf-3926343bfb89}" enabled="0" method="" siteId="{06219a4a-a835-44d5-afaf-3926343bfb89}" removed="1"/>
+  <clbl:label id="{ed006307-e4a9-430f-af16-eea280431306}" enabled="1" method="Standard" siteId="{06219a4a-a835-44d5-afaf-3926343bfb89}" removed="0"/>
 </clbl:labelList>
 </file>
</xml_diff>